<commit_message>
Fix CLI nessages and config
</commit_message>
<xml_diff>
--- a/assets/sample-config.xlsx
+++ b/assets/sample-config.xlsx
@@ -23,7 +23,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="37" uniqueCount="32">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="51" uniqueCount="34">
   <si>
     <t xml:space="preserve">id</t>
   </si>
@@ -68,6 +68,12 @@
   </si>
   <si>
     <t xml:space="preserve">aefl</t>
+  </si>
+  <si>
+    <t xml:space="preserve">auto1</t>
+  </si>
+  <si>
+    <t xml:space="preserve">auto2</t>
   </si>
   <si>
     <t xml:space="preserve">vendor</t>
@@ -361,10 +367,10 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:H2"/>
+  <dimension ref="A1:H4"/>
   <sheetFormatPr defaultColWidth="11.53515625" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="5.07"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="6.12"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="1" width="53.3"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="1" width="21.53"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="1" width="12.15"/>
@@ -424,9 +430,63 @@
         <v>14</v>
       </c>
     </row>
+    <row r="3" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A3" s="1" t="s">
+        <v>15</v>
+      </c>
+      <c r="B3" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="C3" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="D3" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="E3" s="1" t="s">
+        <v>12</v>
+      </c>
+      <c r="F3" s="1" t="n">
+        <v>1244998375585961</v>
+      </c>
+      <c r="G3" s="1" t="s">
+        <v>13</v>
+      </c>
+      <c r="H3" s="1" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="4" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A4" s="1" t="s">
+        <v>16</v>
+      </c>
+      <c r="B4" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="C4" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="D4" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="E4" s="1" t="s">
+        <v>12</v>
+      </c>
+      <c r="F4" s="1" t="n">
+        <v>1244998375585961</v>
+      </c>
+      <c r="G4" s="1" t="s">
+        <v>13</v>
+      </c>
+      <c r="H4" s="1" t="s">
+        <v>14</v>
+      </c>
+    </row>
   </sheetData>
   <hyperlinks>
     <hyperlink ref="B2" r:id="rId1" display="https://www.usaa.com/inet/wc/auto-insurance?vurl=VURL_auto"/>
+    <hyperlink ref="B3" r:id="rId2" display="https://www.usaa.com/inet/wc/auto-insurance?vurl=VURL_auto"/>
+    <hyperlink ref="B4" r:id="rId3" display="https://www.usaa.com/inet/wc/auto-insurance?vurl=VURL_auto"/>
   </hyperlinks>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
   <pageMargins left="0.7875" right="0.7875" top="1.05277777777778" bottom="1.05277777777778" header="0.7875" footer="0.7875"/>
@@ -453,42 +513,42 @@
   <sheetData>
     <row r="1" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>15</v>
+        <v>17</v>
       </c>
       <c r="B1" s="3" t="s">
-        <v>16</v>
+        <v>18</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="1" t="s">
-        <v>17</v>
+        <v>19</v>
       </c>
       <c r="B2" s="4" t="s">
-        <v>18</v>
+        <v>20</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="1" t="s">
-        <v>19</v>
+        <v>21</v>
       </c>
       <c r="B3" s="1" t="s">
-        <v>20</v>
+        <v>22</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="1" t="s">
-        <v>21</v>
+        <v>23</v>
       </c>
       <c r="B4" s="1" t="s">
-        <v>22</v>
+        <v>24</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="1" t="s">
-        <v>23</v>
+        <v>25</v>
       </c>
       <c r="B5" s="1" t="s">
-        <v>24</v>
+        <v>26</v>
       </c>
     </row>
   </sheetData>
@@ -518,26 +578,26 @@
   <sheetData>
     <row r="1" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>15</v>
+        <v>17</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>25</v>
+        <v>27</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="12.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="1" t="s">
-        <v>17</v>
+        <v>19</v>
       </c>
       <c r="B2" s="2" t="s">
-        <v>26</v>
+        <v>28</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="1" t="s">
-        <v>19</v>
+        <v>21</v>
       </c>
       <c r="B3" s="1" t="s">
-        <v>27</v>
+        <v>29</v>
       </c>
     </row>
   </sheetData>
@@ -567,26 +627,26 @@
   <sheetData>
     <row r="1" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>15</v>
+        <v>17</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>28</v>
+        <v>30</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="1" t="s">
-        <v>17</v>
+        <v>19</v>
       </c>
       <c r="B2" s="5" t="s">
-        <v>29</v>
+        <v>31</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="1" t="s">
-        <v>30</v>
+        <v>32</v>
       </c>
       <c r="B3" s="1" t="s">
-        <v>31</v>
+        <v>33</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Restructure for best practice maintainability and distribution
</commit_message>
<xml_diff>
--- a/assets/sample-config.xlsx
+++ b/assets/sample-config.xlsx
@@ -1,6 +1,6 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2">
   <fileVersion appName="Calc"/>
   <workbookPr backupFile="false" showObjects="all" date1904="false"/>
   <workbookProtection/>
@@ -23,7 +23,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="51" uniqueCount="34">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="48" uniqueCount="35">
   <si>
     <t xml:space="preserve">id</t>
   </si>
@@ -55,12 +55,18 @@
     <t xml:space="preserve">https://www.usaa.com/inet/wc/auto-insurance?vurl=VURL_auto</t>
   </si>
   <si>
+    <t xml:space="preserve">[meta]</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ViewContent</t>
+  </si>
+  <si>
+    <t xml:space="preserve">auto1</t>
+  </si>
+  <si>
     <t xml:space="preserve">[meta, google, floodlight]</t>
   </si>
   <si>
-    <t xml:space="preserve">ViewContent</t>
-  </si>
-  <si>
     <t xml:space="preserve">aut-ins</t>
   </si>
   <si>
@@ -68,9 +74,6 @@
   </si>
   <si>
     <t xml:space="preserve">aefl</t>
-  </si>
-  <si>
-    <t xml:space="preserve">auto1</t>
   </si>
   <si>
     <t xml:space="preserve">auto2</t>
@@ -264,37 +267,37 @@
         <a:srgbClr val="000000"/>
       </a:dk1>
       <a:lt1>
-        <a:srgbClr val="ffffff"/>
+        <a:srgbClr val="FFFFFF"/>
       </a:lt1>
       <a:dk2>
         <a:srgbClr val="000000"/>
       </a:dk2>
       <a:lt2>
-        <a:srgbClr val="ffffff"/>
+        <a:srgbClr val="FFFFFF"/>
       </a:lt2>
       <a:accent1>
-        <a:srgbClr val="18a303"/>
+        <a:srgbClr val="18A303"/>
       </a:accent1>
       <a:accent2>
-        <a:srgbClr val="0369a3"/>
+        <a:srgbClr val="0369A3"/>
       </a:accent2>
       <a:accent3>
-        <a:srgbClr val="a33e03"/>
+        <a:srgbClr val="A33E03"/>
       </a:accent3>
       <a:accent4>
-        <a:srgbClr val="8e03a3"/>
+        <a:srgbClr val="8E03A3"/>
       </a:accent4>
       <a:accent5>
-        <a:srgbClr val="c99c00"/>
+        <a:srgbClr val="C99C00"/>
       </a:accent5>
       <a:accent6>
-        <a:srgbClr val="c9211e"/>
+        <a:srgbClr val="C9211E"/>
       </a:accent6>
       <a:hlink>
-        <a:srgbClr val="0000ee"/>
+        <a:srgbClr val="0000EE"/>
       </a:hlink>
       <a:folHlink>
-        <a:srgbClr val="551a8b"/>
+        <a:srgbClr val="551A8B"/>
       </a:folHlink>
     </a:clrScheme>
     <a:fontScheme name="Office">
@@ -368,7 +371,7 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:H4"/>
-  <sheetFormatPr defaultColWidth="11.53515625" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="11.53515625" defaultRowHeight="12.8" customHeight="false" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="6.12"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="1" width="53.3"/>
@@ -417,69 +420,61 @@
       <c r="D2" s="1" t="s">
         <v>11</v>
       </c>
-      <c r="E2" s="1" t="s">
-        <v>12</v>
-      </c>
       <c r="F2" s="1" t="n">
         <v>1244998375585961</v>
       </c>
-      <c r="G2" s="1" t="s">
-        <v>13</v>
-      </c>
-      <c r="H2" s="1" t="s">
-        <v>14</v>
-      </c>
+      <c r="H2" s="1"/>
     </row>
     <row r="3" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="1" t="s">
-        <v>15</v>
+        <v>12</v>
       </c>
       <c r="B3" s="2" t="s">
         <v>9</v>
       </c>
       <c r="C3" s="1" t="s">
-        <v>10</v>
+        <v>13</v>
       </c>
       <c r="D3" s="1" t="s">
         <v>11</v>
       </c>
       <c r="E3" s="1" t="s">
-        <v>12</v>
+        <v>14</v>
       </c>
       <c r="F3" s="1" t="n">
         <v>1244998375585961</v>
       </c>
       <c r="G3" s="1" t="s">
-        <v>13</v>
+        <v>15</v>
       </c>
       <c r="H3" s="1" t="s">
-        <v>14</v>
+        <v>16</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="1" t="s">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="B4" s="2" t="s">
         <v>9</v>
       </c>
       <c r="C4" s="1" t="s">
-        <v>10</v>
+        <v>13</v>
       </c>
       <c r="D4" s="1" t="s">
         <v>11</v>
       </c>
       <c r="E4" s="1" t="s">
-        <v>12</v>
+        <v>14</v>
       </c>
       <c r="F4" s="1" t="n">
         <v>1244998375585961</v>
       </c>
       <c r="G4" s="1" t="s">
-        <v>13</v>
+        <v>15</v>
       </c>
       <c r="H4" s="1" t="s">
-        <v>14</v>
+        <v>16</v>
       </c>
     </row>
   </sheetData>
@@ -504,7 +499,7 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:B5"/>
-  <sheetFormatPr defaultColWidth="11.53515625" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="11.53515625" defaultRowHeight="12.8" customHeight="false" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="12.26"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="1" width="29.77"/>
@@ -513,42 +508,42 @@
   <sheetData>
     <row r="1" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="B1" s="3" t="s">
-        <v>18</v>
+        <v>19</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="1" t="s">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="B2" s="4" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="1" t="s">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="B3" s="1" t="s">
-        <v>22</v>
+        <v>23</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="1" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="B4" s="1" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="1" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="B5" s="1" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
     </row>
   </sheetData>
@@ -571,33 +566,33 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:B3"/>
-  <sheetFormatPr defaultColWidth="11.53515625" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="11.53515625" defaultRowHeight="12.8" customHeight="false" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="1" width="25.48"/>
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="12.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="1" t="s">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="B2" s="2" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="1" t="s">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="B3" s="1" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
     </row>
   </sheetData>
@@ -620,33 +615,33 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:B3"/>
-  <sheetFormatPr defaultColWidth="11.53515625" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="11.53515625" defaultRowHeight="12.8" customHeight="false" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="1" width="18.89"/>
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="1" t="s">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="B2" s="5" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="1" t="s">
-        <v>32</v>
+        <v>33</v>
       </c>
       <c r="B3" s="1" t="s">
-        <v>33</v>
+        <v>34</v>
       </c>
     </row>
   </sheetData>

</xml_diff>